<commit_message>
Több napos események és szálláskérés
- Esemény: új „Utolsó nap” mező (több napos esemény); megjelenik a listákban, az értesítésekben,
  a riportban és a naptár-feliratkozásban; import táblázatból („Utolsó nap”) és Google Naptárból
- Szálláskérés: csak Nyíregyházán kívüli, több napos eseménynél engedélyezhető (új eseménynél
  alapból be van kapcsolva); a tag a „Részt veszek”/„Talán” válasz mellé bepipálhatja, hogy
  „Kérek szállást”; „Nem” válasznál törlődik
- Admin: szálláskérők száma és oszlop a követő nézetben; „Szállást kér” oszlop és összesítő
  a riportban (Excel, CSV, nyomtatás, e-mail)
- Importsablon: „Utolsó nap” és „Szálláskérés” oszlop
- Tesztek, README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqK5QRU9YGqtKeGywQEwCy
</commit_message>
<xml_diff>
--- a/templates/esemenyek_import_sablon.xlsx
+++ b/templates/esemenyek_import_sablon.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="65">
   <si>
     <t>Esemény neve</t>
   </si>
@@ -20,6 +20,9 @@
     <t>Dátum</t>
   </si>
   <si>
+    <t>Utolsó nap</t>
+  </si>
+  <si>
     <t>Kezdés</t>
   </si>
   <si>
@@ -35,6 +38,9 @@
     <t>Turné</t>
   </si>
   <si>
+    <t>Szálláskérés</t>
+  </si>
+  <si>
     <t>Ország</t>
   </si>
   <si>
@@ -59,6 +65,9 @@
     <t>2026-11-03</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>18:00</t>
   </si>
   <si>
@@ -89,9 +98,6 @@
     <t>2026-10-31</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Adventi koncert – főpróba</t>
   </si>
   <si>
@@ -131,15 +137,21 @@
     <t>Fellépő ruha: fekete</t>
   </si>
   <si>
-    <t>Indulás Bécsbe</t>
+    <t>Bécsi turné</t>
   </si>
   <si>
     <t>2027-03-12</t>
   </si>
   <si>
+    <t>2027-03-15</t>
+  </si>
+  <si>
     <t>07:00</t>
   </si>
   <si>
+    <t>20:00</t>
+  </si>
+  <si>
     <t>utazás</t>
   </si>
   <si>
@@ -149,7 +161,10 @@
     <t>igen</t>
   </si>
   <si>
-    <t>Iskola, parkoló</t>
+    <t>Ausztria</t>
+  </si>
+  <si>
+    <t>Bécs</t>
   </si>
   <si>
     <t>2027-02-20</t>
@@ -174,6 +189,12 @@
   </si>
   <si>
     <t>Turné: „igen”, ha az esemény koncertturné része.</t>
+  </si>
+  <si>
+    <t>Utolsó nap: csak több napos eseménynél kell kitölteni (ÉÉÉÉ-HH-NN).</t>
+  </si>
+  <si>
+    <t>Szálláskérés: „igen” vagy „nem” – a tagok kérhetnek-e szállást. Csak Nyíregyházán kívüli, több napos eseménynél lehetséges; üresen hagyva ilyenkor automatikusan engedélyezett.</t>
   </si>
   <si>
     <t>Visszajelzési határidő: ha üresen hagyod, az import ablakban megadott számú nappal az esemény előtt lesz.</t>
@@ -580,24 +601,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9" style="1" customWidth="1"/>
-    <col min="4" max="5" width="10" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8" style="1" customWidth="1"/>
-    <col min="8" max="8" width="12" style="1" customWidth="1"/>
-    <col min="9" max="9" width="14" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26" style="1" customWidth="1"/>
-    <col min="11" max="11" width="24" style="1" customWidth="1"/>
-    <col min="12" max="12" width="22" style="1" customWidth="1"/>
-    <col min="13" max="13" width="30" style="1" customWidth="1"/>
+    <col min="2" max="3" width="12" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9" style="1" customWidth="1"/>
+    <col min="5" max="6" width="10" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8" style="1" customWidth="1"/>
+    <col min="9" max="9" width="13" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14" style="1" customWidth="1"/>
+    <col min="12" max="12" width="26" style="1" customWidth="1"/>
+    <col min="13" max="13" width="24" style="1" customWidth="1"/>
+    <col min="14" max="14" width="22" style="1" customWidth="1"/>
+    <col min="15" max="15" width="30" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -637,169 +659,199 @@
       <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="J2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" s="1" t="s">
+      <c r="F3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="I3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="L3" s="1" t="s">
         <v>33</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>33</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="L5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="M5" s="1" t="s">
-        <v>47</v>
+        <v>34</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -810,7 +862,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -818,52 +870,62 @@
   <sheetData>
     <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>57</v>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Eseményimport: „Van főpróbája” oszlop – a főpróba automatikus létrehozása
„igen” esetén az import a koncert előtti napra, a koncert kezdési idejében,
2 órás főpróbát hoz létre ugyanott, és a koncerthez kapcsolja; „nem” esetén
a koncert nem kapcsolódik automatikusan más főpróbához. Üresen a korábbi
működés marad. Korábban beimportált piszkozat koncert újraimportáláskor
megkapja a főpróbáját.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqK5QRU9YGqtKeGywQEwCy
</commit_message>
<xml_diff>
--- a/templates/esemenyek_import_sablon.xlsx
+++ b/templates/esemenyek_import_sablon.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="69">
   <si>
     <t>Esemény neve</t>
   </si>
@@ -32,6 +32,9 @@
     <t>Típus</t>
   </si>
   <si>
+    <t>Van főpróbája</t>
+  </si>
+  <si>
     <t>Énekkar</t>
   </si>
   <si>
@@ -137,6 +140,15 @@
     <t>Fellépő ruha: fekete</t>
   </si>
   <si>
+    <t>Újévi koncert</t>
+  </si>
+  <si>
+    <t>2027-01-09</t>
+  </si>
+  <si>
+    <t>igen</t>
+  </si>
+  <si>
     <t>Bécsi turné</t>
   </si>
   <si>
@@ -158,9 +170,6 @@
     <t>Pro Musica</t>
   </si>
   <si>
-    <t>igen</t>
-  </si>
-  <si>
     <t>Ausztria</t>
   </si>
   <si>
@@ -200,7 +209,10 @@
     <t>Visszajelzési határidő: ha üresen hagyod, az import ablakban megadott számú nappal az esemény előtt lesz.</t>
   </si>
   <si>
-    <t>A koncertek automatikusan a legközelebbi (14 napon belüli) főpróbához kapcsolódnak – ez az appban módosítható.</t>
+    <t>Van főpróbája (csak koncertnél): „igen” esetén az app létrehozza a főpróbát is – alapból a koncert előtti napon, a koncert kezdési idejében, 2 órásat, ugyanott és ugyanannak a kórusnak –, és hozzákapcsolja a koncerthez. „nem” esetén a koncertnek nincs főpróbája.</t>
+  </si>
+  <si>
+    <t>Ha üresen hagyod, a koncert a legközelebbi (14 napon belüli) főpróbához kapcsolódik – így a főpróbát külön sorban is megadhatod. Az appban mindez módosítható.</t>
   </si>
   <si>
     <t>Az importált események piszkozatként jönnek létre: ellenőrzés után az appban kell közzétenni őket.</t>
@@ -601,25 +613,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" style="1" customWidth="1"/>
     <col min="2" max="3" width="12" style="1" customWidth="1"/>
     <col min="4" max="4" width="9" style="1" customWidth="1"/>
     <col min="5" max="6" width="10" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20" style="1" customWidth="1"/>
-    <col min="8" max="8" width="8" style="1" customWidth="1"/>
-    <col min="9" max="9" width="13" style="1" customWidth="1"/>
-    <col min="10" max="10" width="12" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="26" style="1" customWidth="1"/>
-    <col min="13" max="13" width="24" style="1" customWidth="1"/>
-    <col min="14" max="14" width="22" style="1" customWidth="1"/>
-    <col min="15" max="15" width="30" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14" style="1" customWidth="1"/>
+    <col min="8" max="8" width="20" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8" style="1" customWidth="1"/>
+    <col min="10" max="10" width="13" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12" style="1" customWidth="1"/>
+    <col min="12" max="12" width="14" style="1" customWidth="1"/>
+    <col min="13" max="13" width="26" style="1" customWidth="1"/>
+    <col min="14" max="14" width="24" style="1" customWidth="1"/>
+    <col min="15" max="15" width="22" style="1" customWidth="1"/>
+    <col min="16" max="16" width="30" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -665,37 +678,40 @@
       <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>24</v>
@@ -710,45 +726,48 @@
         <v>27</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>34</v>
@@ -757,45 +776,48 @@
         <v>35</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>34</v>
@@ -804,42 +826,45 @@
         <v>35</v>
       </c>
       <c r="O4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="H5" s="1" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="L5" s="1" t="s">
         <v>25</v>
@@ -848,10 +873,63 @@
         <v>34</v>
       </c>
       <c r="N5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="I6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -862,7 +940,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -870,62 +948,67 @@
   <sheetData>
     <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>